<commit_message>
Fixed Check type success rate calculation
</commit_message>
<xml_diff>
--- a/Experiment results and Raw Data/Trolley/Tests_Trolley_with_Summary.xlsx
+++ b/Experiment results and Raw Data/Trolley/Tests_Trolley_with_Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\Desktop\Master Thesis\Experiment results and Raw Data\Trolley\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E302F76-6F92-49FF-A3E7-96B9EE4B21D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ABBFC0A-BE2C-4B22-AFF6-29E233109851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Event_logs!$A$1:$A$1588</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Handnotes!$A$1:$A$95</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10161" uniqueCount="2169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10160" uniqueCount="2169">
   <si>
     <t>count (y/n)</t>
   </si>
@@ -6784,7 +6785,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -6905,12 +6906,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
@@ -9452,9 +9452,7 @@
       <c r="F37" s="53" t="s">
         <v>2148</v>
       </c>
-      <c r="G37" s="25" t="s">
-        <v>19</v>
-      </c>
+      <c r="G37" s="25"/>
       <c r="H37" s="25"/>
       <c r="I37" s="25"/>
       <c r="J37" s="6"/>
@@ -10813,7 +10811,7 @@
       </c>
       <c r="G79" s="33">
         <f>COUNTIF(G2:G66,"correct")</f>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H79" s="35" t="s">
         <v>60</v>
@@ -11155,6 +11153,7 @@
       <c r="AW95"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A95" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -55500,32 +55499,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="72" t="s">
         <v>2057</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
+      <c r="Q1" s="72"/>
+      <c r="R1" s="72"/>
+      <c r="S1" s="72"/>
+      <c r="T1" s="72"/>
+      <c r="U1" s="72"/>
+      <c r="V1" s="72"/>
+      <c r="W1" s="72"/>
+      <c r="X1" s="72"/>
       <c r="Y1" s="37"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
@@ -55863,7 +55862,7 @@
       <c r="A10" t="s">
         <v>2081</v>
       </c>
-      <c r="B10" s="72">
+      <c r="B10">
         <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$K$2:$K$95,"YES")</f>
         <v>24</v>
       </c>
@@ -55871,7 +55870,7 @@
         <f>COUNTIF(Handnotes!$A$2:$A$95,"y")</f>
         <v>53</v>
       </c>
-      <c r="D10" s="73">
+      <c r="D10" s="71">
         <f>B10/C10</f>
         <v>0.45283018867924529</v>
       </c>
@@ -55895,7 +55894,7 @@
       <c r="A11" t="s">
         <v>2167</v>
       </c>
-      <c r="B11" s="71">
+      <c r="B11" s="70">
         <f>COUNTIFS(Handnotes!$J$2:$J$95,"success",Handnotes!$K$2:$K$95,"YES")</f>
         <v>18</v>
       </c>
@@ -55903,7 +55902,7 @@
         <f>B10</f>
         <v>24</v>
       </c>
-      <c r="D11" s="73">
+      <c r="D11" s="71">
         <f>B11/C11</f>
         <v>0.75</v>
       </c>
@@ -55933,7 +55932,7 @@
       </c>
       <c r="B13" s="45">
         <f ca="1">NOW()</f>
-        <v>46216.791535879631</v>
+        <v>46218.570535763887</v>
       </c>
       <c r="C13" t="str">
         <f>""</f>
@@ -56173,11 +56172,11 @@
         <v>2163</v>
       </c>
       <c r="I18">
-        <f>COUNTIF(C26:C90,"Laundry Trolley")</f>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$D$2:$D$95,"Laundry Trolley")</f>
         <v>19</v>
       </c>
       <c r="J18">
-        <f>COUNTIFS(E26:E90, "correct",C26:C90,"Laundry Trolley")</f>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$G$2:$G$95, "correct",Handnotes!$D$2:$D$95,"Laundry Trolley")</f>
         <v>19</v>
       </c>
       <c r="K18" s="69">
@@ -56234,12 +56233,12 @@
         <v>2164</v>
       </c>
       <c r="I19">
-        <f>COUNTIF(C27:C91,"Trash Trolley")</f>
-        <v>18</v>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$D$2:$D$95,"Trash Trolley")</f>
+        <v>19</v>
       </c>
       <c r="J19">
-        <f>COUNTIFS(E27:E91, "correct",C27:C91,"Trash Trolley")</f>
-        <v>18</v>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$G$2:$G$95, "correct",Handnotes!$D$2:$D$95,"Trash Trolley")</f>
+        <v>19</v>
       </c>
       <c r="K19" s="69">
         <f t="shared" ref="K19:K21" si="5">J19/I19</f>
@@ -56273,11 +56272,11 @@
         <v>2165</v>
       </c>
       <c r="I20">
-        <f>COUNTIF(C28:C92,"empty")</f>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$D$2:$D$95,"empty")</f>
         <v>15</v>
       </c>
       <c r="J20">
-        <f>COUNTIFS(E28:E92, "correct",C28:C92,"empty")</f>
+        <f>COUNTIFS(Handnotes!$A$2:$A$95,"y",Handnotes!$G$2:$G$95, "correct",Handnotes!$D$2:$D$95,"empty")</f>
         <v>14</v>
       </c>
       <c r="K20" s="69">
@@ -56313,15 +56312,15 @@
       </c>
       <c r="I21">
         <f>SUM(I18:I20)</f>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J21">
         <f>SUM(J18:J20)</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="5"/>
-        <v>0.98076923076923073</v>
+        <v>0.98113207547169812</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">

</xml_diff>